<commit_message>
feat: implement stock transfer module with database schema, controller logic, and bulk upload interface
</commit_message>
<xml_diff>
--- a/public/assets/templates/excel/template_inventory_upload_susut_simpan.xlsx
+++ b/public/assets/templates/excel/template_inventory_upload_susut_simpan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\project_warehouse\public\assets\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF275B4-8006-4364-A792-CEBD5A5607C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F6F4982-FBA5-44D1-BBDF-A89AA5867039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{597B7802-D5FA-46AC-AF8D-9346B9AC7C46}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>UOM</t>
   </si>
@@ -76,6 +76,21 @@
   </si>
   <si>
     <t>%_SUSUT_SIMPAN</t>
+  </si>
+  <si>
+    <t>TGL_BA</t>
+  </si>
+  <si>
+    <t>MATDOC_SCRAP</t>
+  </si>
+  <si>
+    <t>MATDOC_YEAR</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>NO_BA</t>
   </si>
 </sst>
 </file>
@@ -473,78 +488,97 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E674FD-0AB5-4C99-8A62-7683B95A16AC}">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.54296875" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.6328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:22" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>